<commit_message>
Amazon Price Tracker - All tests passing - CODETESTERS
</commit_message>
<xml_diff>
--- a/testdata/PriceData.xlsx
+++ b/testdata/PriceData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
   <si>
     <t>S.No</t>
   </si>
@@ -32,10 +32,10 @@
     <t>Timestamp</t>
   </si>
   <si>
-    <t>Aquaguard Delight Aquasaver RO+UV+UF+MC Tech | 2-year filter life | With Mega Sediment filter | 2 Free cleaning service ...</t>
-  </si>
-  <si>
-    <t>₹11,499</t>
+    <t>Native M1 Pro Water Purifier by Urban Company | Smart Real-Time Tracking | 10-Stage RO+UV+Copper+Alkaline+Mineraliser | ...</t>
+  </si>
+  <si>
+    <t>₹17,499</t>
   </si>
   <si>
     <t>—</t>
@@ -44,19 +44,19 @@
     <t>Initial</t>
   </si>
   <si>
-    <t>04-Jun 12:59</t>
-  </si>
-  <si>
-    <t>Native M1 Pro Water Purifier by Urban Company | Smart Real-Time Tracking | 10-Stage RO+UV+Copper+Alkaline+Mineraliser | ...</t>
-  </si>
-  <si>
-    <t>₹17,499</t>
-  </si>
-  <si>
-    <t>Pureit Classic 23 L Gravity Based Water Purifier | Activated Carbon Filtration | No Electricity Required | Multi-Stage P...</t>
-  </si>
-  <si>
-    <t>₹3,299</t>
+    <t>04-Jun 13:21</t>
+  </si>
+  <si>
+    <t>Native M0 Water Purifier by Urban Company | 8-Stage RO+UV+Mineraliser | No Service for 2 Years | India’s Only 2-Year Unc...</t>
+  </si>
+  <si>
+    <t>₹13,499</t>
+  </si>
+  <si>
+    <t>AQUA D PURE 4 in 1 Copper RO Water Purifier with 10 Stage Purification Filtration, UV, UF, TDS Adjuster and 12 Liter Lar...</t>
+  </si>
+  <si>
+    <t>₹5,248</t>
   </si>
   <si>
     <t>AquaX Pure Ro water Purifier RO+UV+COPPER+ZINC 10 Stages Purification. Advance MTDS and HTDS Membrane, Suitable for all ...</t>
@@ -65,16 +65,10 @@
     <t>₹4,999</t>
   </si>
   <si>
-    <t>AQUA D PURE 4 in 1 Copper RO Water Purifier with 10 Stage Purification Filtration, UV, UF, TDS Adjuster and 12 Liter Lar...</t>
-  </si>
-  <si>
-    <t>₹5,248</t>
-  </si>
-  <si>
-    <t>No Change</t>
-  </si>
-  <si>
-    <t>04-Jun 13:01</t>
+    <t>Aquaguard Delight NXT Aquasaver 9-Stage Water Purifier | Upto 60% Water Savings | RO+UV+UF+MC Tech | Suitable for Borewe...</t>
+  </si>
+  <si>
+    <t>₹10,499</t>
   </si>
 </sst>
 </file>
@@ -82,7 +76,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="2">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -95,30 +89,6 @@
       <sz val="11.0"/>
       <b val="true"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="53"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="53"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="53"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="53"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -168,21 +138,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="true"/>
   </cellXfs>
 </styleSheet>
@@ -234,11 +196,11 @@
       <c r="D2" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="E2" t="s" s="8">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s" s="8">
-        <v>20</v>
+      <c r="E2" t="s" s="2">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -254,11 +216,11 @@
       <c r="D3" t="s" s="3">
         <v>8</v>
       </c>
-      <c r="E3" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s" s="10">
-        <v>20</v>
+      <c r="E3" t="s" s="3">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s" s="3">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -294,11 +256,11 @@
       <c r="D5" t="s" s="5">
         <v>8</v>
       </c>
-      <c r="E5" t="s" s="14">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s" s="14">
-        <v>20</v>
+      <c r="E5" t="s" s="5">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s" s="5">
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -314,11 +276,11 @@
       <c r="D6" t="s" s="6">
         <v>8</v>
       </c>
-      <c r="E6" t="s" s="12">
-        <v>19</v>
-      </c>
-      <c r="F6" t="s" s="12">
-        <v>20</v>
+      <c r="E6" t="s" s="6">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s" s="6">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>